<commit_message>
feat: complete workspace roadmap through S6-15
</commit_message>
<xml_diff>
--- a/src-tauri/tests/fixtures/workbook/compatibility-baseline.xlsx
+++ b/src-tauri/tests/fixtures/workbook/compatibility-baseline.xlsx
@@ -9,13 +9,39 @@
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Details" sheetId="2" r:id="rId2"/>
+    <sheet name="Inventory" sheetId="3" r:id="rId3"/>
+    <sheet name="Protected" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Details!$A$1:$B$2</definedName>
+    <definedName name="AmountRange">Summary!$B$2:$B$2</definedName>
+    <definedName name="Codes" localSheetId="1">Details!$A$2:$A$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Summary!$A$1:$F$5</definedName>
+    <definedName name="ReportWindow">Summary!$A$1:$F$4</definedName>
+    <definedName name="TaxRate">0.13</definedName>
+    <definedName name="TeamLabel">"R&amp;D"</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <externalReferences>
+    <externalReference r:id="rIdExternalFixture"/>
+  </externalReferences>
+  <pivotCaches>
+    <pivotCache cacheId="1" r:id="rIdPivotCacheFixture"/>
+  </pivotCaches>
+  <workbookProtection lockStructure="1" workbookPassword="ABCD"/>
 </workbook>
 </file>
 
+<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <connection id="7" name="Warehouse fixture" type="5" refreshOnLoad="1" background="0" saveData="1">
+    <dbPr connection="Server=secret.example;Password=not-for-ui" command="SELECT 1"/>
+  </connection>
+</connections>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Item</t>
   </si>
@@ -26,27 +52,74 @@
     <t>Approved</t>
   </si>
   <si>
+    <t>Due date</t>
+  </si>
+  <si>
+    <t>Reviewed at</t>
+  </si>
+  <si>
+    <t>Formula error</t>
+  </si>
+  <si>
     <t>Alpha</t>
   </si>
   <si>
     <t>Total</t>
   </si>
   <si>
+    <t>Named total</t>
+  </si>
+  <si>
     <t>Merged fixture title</t>
   </si>
   <si>
     <t>Code</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>A-001</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Hardware</t>
+  </si>
+  <si>
+    <t>Notebook</t>
+  </si>
+  <si>
+    <t>Stationery</t>
+  </si>
+  <si>
+    <t>Locked content</t>
+  </si>
+  <si>
+    <t>Read-only fixture</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -91,17 +164,253 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Inventory stock</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Stock</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Inventory!$A$2:$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Keyboard</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Notebook</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Inventory!$B$2:$B$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Inventory marker"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2438400" y="3429000"/>
+          <a:ext cx="9525" cy="9525"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="InventoryStockChart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <externalBook r:id="rId1">
+    <sheetNames>
+      <sheetName val="ExternalData"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:C3" sheet="Inventory"/>
+  </cacheSource>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="InventoryPivot" cacheId="1"/>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
+  <slicer name="CategorySlicer" cache="CategorySlicerCache"/>
+</slicers>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InventoryTable" displayName="InventoryTable" ref="A1:C3" totalsRowShown="0">
+  <autoFilter ref="A1:C3"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Product"/>
+    <tableColumn id="2" name="Stock"/>
+    <tableColumn id="3" name="Category"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -389,14 +698,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -406,10 +718,19 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="27.75" customHeight="1">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2">
         <v>1250.5</v>
@@ -417,19 +738,38 @@
       <c r="C2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" s="3">
+        <v>46223</v>
+      </c>
+      <c r="E2" s="4">
+        <v>46223.60434027778</v>
+      </c>
+      <c r="F2" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <f>SUM(B2:B2)</f>
         <v>1250.5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <f>SUM(AmountRange)</f>
+        <v>1250.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -438,26 +778,120 @@
   <mergeCells count="1">
     <mergeCell ref="A5:C5"/>
   </mergeCells>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1" headings="1" gridLines="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="200" verticalDpi="200"/>
+  <headerFooter>
+    <oddHeader>&amp;LConfidential&amp;CQuarterly summary&amp;RPage &amp;P of &amp;N</oddHeader>
+    <oddFooter>&amp;CGenerated by LongEdit fixture</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B2"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid status" error="Use Active, Paused, or Closed" promptTitle="Status" prompt="Choose an approved status" sqref="B2:B101">
+      <formula1>"Active,Paused,Closed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+  <pivotTableParts count="1">
+    <pivotTablePart r:id="rIdPivotFixture"/>
+  </pivotTableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection password="B459" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete formula theme and pivot audit stages
</commit_message>
<xml_diff>
--- a/src-tauri/tests/fixtures/workbook/compatibility-baseline.xlsx
+++ b/src-tauri/tests/fixtures/workbook/compatibility-baseline.xlsx
@@ -384,15 +384,63 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdRecords" recordCount="2" refreshOnLoad="1">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:C3" sheet="Inventory"/>
   </cacheSource>
+  <cacheFields count="3">
+    <cacheField name="Product">
+      <sharedItems containsString="1" count="2">
+        <s v="Keyboard"/>
+        <s v="Notebook"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Stock">
+      <sharedItems containsNumber="1" count="2" minValue="12" maxValue="30"/>
+    </cacheField>
+    <cacheField name="Category">
+      <sharedItems containsString="1" count="2">
+        <s v="Hardware"/>
+        <s v="Stationery"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2">
+  <r>
+    <x v="0"/>
+    <n v="12"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="30"/>
+    <x v="1"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="InventoryPivot" cacheId="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="InventoryPivot" cacheId="1">
+  <location ref="E2:G6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" showAll="0"/>
+    <pivotField axis="axisCol" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <dataFields count="1">
+    <dataField name="Sum of Stock" fld="1" subtotal="sum"/>
+  </dataFields>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>